<commit_message>
with itr1,2,3 pics and eval templates
</commit_message>
<xml_diff>
--- a/grid-chat-streamlit/test/iteration2_rough_plan.xlsx
+++ b/grid-chat-streamlit/test/iteration2_rough_plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\problem_first_ai\capstore16_code\unblocking_icq_phase1\grid-chat-streamlit\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{60162568-28CE-410A-8719-9223A941C5A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{F4FE69B0-FCB6-41DA-8EE4-AF55B397464B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{DAA4B09E-5322-4E17-914F-81B6FCADEE0B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{DAA4B09E-5322-4E17-914F-81B6FCADEE0B}"/>
   </bookViews>
   <sheets>
     <sheet name="Recommended_Tools" sheetId="1" r:id="rId1"/>
@@ -1389,6 +1389,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FB89FC5-5825-4B29-AD29-515F36822684}">
   <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.36328125" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" customWidth="1"/>
+    <col min="3" max="3" width="32.1796875" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="6" max="6" width="15.26953125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -1410,7 +1417,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>27</v>
       </c>
@@ -1430,7 +1437,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>27</v>
       </c>
@@ -1450,7 +1457,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>27</v>
       </c>
@@ -1470,7 +1477,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>27</v>
       </c>
@@ -1490,7 +1497,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>44</v>
       </c>
@@ -1510,7 +1517,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>44</v>
       </c>
@@ -1530,7 +1537,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>44</v>
       </c>
@@ -1550,7 +1557,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>44</v>
       </c>
@@ -1570,7 +1577,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="116" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>58</v>
       </c>
@@ -1590,7 +1597,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>58</v>
       </c>
@@ -1610,7 +1617,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>65</v>
       </c>
@@ -1630,7 +1637,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>65</v>
       </c>
@@ -1650,7 +1657,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>65</v>
       </c>
@@ -1670,7 +1677,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>75</v>
       </c>
@@ -1690,7 +1697,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>75</v>
       </c>
@@ -1710,7 +1717,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>75</v>
       </c>
@@ -1730,7 +1737,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>75</v>
       </c>
@@ -1750,7 +1757,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>88</v>
       </c>
@@ -1770,7 +1777,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>88</v>
       </c>
@@ -1790,7 +1797,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>95</v>
       </c>
@@ -1810,7 +1817,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>95</v>
       </c>
@@ -1830,7 +1837,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="87" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>95</v>
       </c>
@@ -1850,7 +1857,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>105</v>
       </c>
@@ -1870,7 +1877,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>105</v>
       </c>
@@ -1890,7 +1897,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
         <v>105</v>
       </c>
@@ -1910,7 +1917,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>12</v>
       </c>
@@ -1930,7 +1937,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="58" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
         <v>12</v>
       </c>

</xml_diff>